<commit_message>
csv excel parsing notebooks added
</commit_message>
<xml_diff>
--- a/data/raw/structured_files/inventory.xlsx
+++ b/data/raw/structured_files/inventory.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,31 +414,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -568,6 +556,121 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>1080p webcam with noise cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Headphones</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="D7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Over-ear wireless headphones with active noise cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>All-in-one wireless printer with scanner and copier</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>USB Hub</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="D9" t="n">
+        <v>300</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>7-port USB 3.0 hub with fast data transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>External SSD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>129.99</v>
+      </c>
+      <c r="D10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1TB portable external SSD with USB-C connectivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Router</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>89.98999999999999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>60</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Dual-band Wi-Fi 6 router with mesh support</t>
         </is>
       </c>
     </row>
@@ -586,17 +689,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Total_Items</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total_Value</t>
         </is>
@@ -605,27 +708,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>1389.97</v>
+        <v>284.96</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>109.98</v>
+        <v>1809.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>